<commit_message>
Feat: Finalized PCB and added V1 and V2 of the Casing
</commit_message>
<xml_diff>
--- a/hardware/BodyTempSens_Data.xlsx
+++ b/hardware/BodyTempSens_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daanheetkamp/Desktop/BodyTempSensor/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daanheetkamp/Desktop/heart-heat-sensor/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFC80BE-FF6D-F947-A5FA-7AEC4A821F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A290EE3-9C77-A740-B64B-26226019A371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="28200" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="4" r:id="rId1"/>
@@ -3363,16 +3363,10 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3384,14 +3378,20 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3402,7 +3402,207 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
           <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3466,6 +3666,158 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
           <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
@@ -3491,6 +3843,62 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
           <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3538,7 +3946,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3554,7 +3962,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3602,7 +4010,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3618,7 +4026,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3659,414 +4067,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
           <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4756,15 +4756,15 @@
 </file>
 
 <file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="LCSC__WM2212110099_20260617034224" connectionId="2" xr16:uid="{06E6BE92-5986-4143-9189-C64D0AAC269F}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="LCSC__WM2407090249_20260617034145" connectionId="3" xr16:uid="{9F228B63-54CA-1A4A-9361-CAB5D71DFF0A}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="LCSC__WM2407090249_20260617034145" connectionId="3" xr16:uid="{9F228B63-54CA-1A4A-9361-CAB5D71DFF0A}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="LCSC__WM2509140097_20260617034302_1" connectionId="4" xr16:uid="{636388EF-35EB-4340-B01C-0AE102A00007}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="LCSC__WM2509140097_20260617034302_1" connectionId="4" xr16:uid="{636388EF-35EB-4340-B01C-0AE102A00007}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="LCSC__WM2212110099_20260617034224" connectionId="2" xr16:uid="{06E6BE92-5986-4143-9189-C64D0AAC269F}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6988,30 +6988,30 @@
       <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="49" t="s">
+      <c r="N1" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="O1" s="49"/>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="49"/>
-      <c r="R1" s="49"/>
-      <c r="S1" s="49"/>
-      <c r="T1" s="49"/>
-      <c r="U1" s="49"/>
-      <c r="V1" s="49"/>
-      <c r="W1" s="49"/>
-      <c r="Y1" s="49" t="s">
+      <c r="O1" s="58"/>
+      <c r="P1" s="58"/>
+      <c r="Q1" s="58"/>
+      <c r="R1" s="58"/>
+      <c r="S1" s="58"/>
+      <c r="T1" s="58"/>
+      <c r="U1" s="58"/>
+      <c r="V1" s="58"/>
+      <c r="W1" s="58"/>
+      <c r="Y1" s="58" t="s">
         <v>223</v>
       </c>
-      <c r="Z1" s="49"/>
-      <c r="AA1" s="49"/>
-      <c r="AB1" s="49"/>
-      <c r="AC1" s="49"/>
-      <c r="AD1" s="49"/>
-      <c r="AE1" s="49"/>
-      <c r="AF1" s="49"/>
-      <c r="AG1" s="49"/>
-      <c r="AH1" s="49"/>
+      <c r="Z1" s="58"/>
+      <c r="AA1" s="58"/>
+      <c r="AB1" s="58"/>
+      <c r="AC1" s="58"/>
+      <c r="AD1" s="58"/>
+      <c r="AE1" s="58"/>
+      <c r="AF1" s="58"/>
+      <c r="AG1" s="58"/>
+      <c r="AH1" s="58"/>
     </row>
     <row r="2" spans="1:47" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -7270,10 +7270,10 @@
       <c r="AH5" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="AJ5" s="56" t="s">
+      <c r="AJ5" s="49" t="s">
         <v>226</v>
       </c>
-      <c r="AK5" s="57"/>
+      <c r="AK5" s="50"/>
       <c r="AM5" t="s">
         <v>233</v>
       </c>
@@ -7694,24 +7694,24 @@
         <f>Y13*AB13</f>
         <v>0.39599999999999996</v>
       </c>
-      <c r="AE13" s="53" t="s">
+      <c r="AE13" s="51" t="s">
         <v>211</v>
       </c>
-      <c r="AF13" s="54"/>
-      <c r="AG13" s="54"/>
-      <c r="AH13" s="54"/>
-      <c r="AI13" s="54"/>
-      <c r="AJ13" s="54"/>
-      <c r="AK13" s="55"/>
-      <c r="AO13" s="53" t="s">
+      <c r="AF13" s="52"/>
+      <c r="AG13" s="52"/>
+      <c r="AH13" s="52"/>
+      <c r="AI13" s="52"/>
+      <c r="AJ13" s="52"/>
+      <c r="AK13" s="53"/>
+      <c r="AO13" s="51" t="s">
         <v>211</v>
       </c>
-      <c r="AP13" s="54"/>
-      <c r="AQ13" s="54"/>
-      <c r="AR13" s="54"/>
-      <c r="AS13" s="54"/>
-      <c r="AT13" s="54"/>
-      <c r="AU13" s="55"/>
+      <c r="AP13" s="52"/>
+      <c r="AQ13" s="52"/>
+      <c r="AR13" s="52"/>
+      <c r="AS13" s="52"/>
+      <c r="AT13" s="52"/>
+      <c r="AU13" s="53"/>
     </row>
     <row r="14" spans="1:47" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="P14" s="4">
@@ -7732,28 +7732,28 @@
         <v>0.86</v>
       </c>
       <c r="AC14" s="4"/>
-      <c r="AE14" s="50" t="s">
+      <c r="AE14" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="AF14" s="51"/>
-      <c r="AG14" s="58"/>
+      <c r="AF14" s="55"/>
+      <c r="AG14" s="56"/>
       <c r="AH14" s="13"/>
-      <c r="AI14" s="50" t="s">
+      <c r="AI14" s="54" t="s">
         <v>212</v>
       </c>
-      <c r="AJ14" s="51"/>
-      <c r="AK14" s="52"/>
-      <c r="AO14" s="50" t="s">
+      <c r="AJ14" s="55"/>
+      <c r="AK14" s="57"/>
+      <c r="AO14" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="AP14" s="51"/>
-      <c r="AQ14" s="58"/>
+      <c r="AP14" s="55"/>
+      <c r="AQ14" s="56"/>
       <c r="AR14" s="13"/>
-      <c r="AS14" s="50" t="s">
+      <c r="AS14" s="54" t="s">
         <v>212</v>
       </c>
-      <c r="AT14" s="51"/>
-      <c r="AU14" s="52"/>
+      <c r="AT14" s="55"/>
+      <c r="AU14" s="57"/>
     </row>
     <row r="15" spans="1:47" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="I15" t="s">
@@ -7876,50 +7876,50 @@
         <f>J8-(J13/2)</f>
         <v>1.1308825454545455</v>
       </c>
-      <c r="AE19" s="53" t="s">
+      <c r="AE19" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="AF19" s="54"/>
-      <c r="AG19" s="54"/>
-      <c r="AH19" s="54"/>
-      <c r="AI19" s="54"/>
-      <c r="AJ19" s="54"/>
-      <c r="AK19" s="55"/>
-      <c r="AO19" s="53" t="s">
+      <c r="AF19" s="52"/>
+      <c r="AG19" s="52"/>
+      <c r="AH19" s="52"/>
+      <c r="AI19" s="52"/>
+      <c r="AJ19" s="52"/>
+      <c r="AK19" s="53"/>
+      <c r="AO19" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="AP19" s="54"/>
-      <c r="AQ19" s="54"/>
-      <c r="AR19" s="54"/>
-      <c r="AS19" s="54"/>
-      <c r="AT19" s="54"/>
-      <c r="AU19" s="55"/>
+      <c r="AP19" s="52"/>
+      <c r="AQ19" s="52"/>
+      <c r="AR19" s="52"/>
+      <c r="AS19" s="52"/>
+      <c r="AT19" s="52"/>
+      <c r="AU19" s="53"/>
     </row>
     <row r="20" spans="6:47" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-      <c r="AE20" s="50" t="s">
+      <c r="AE20" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="AF20" s="51"/>
-      <c r="AG20" s="58"/>
+      <c r="AF20" s="55"/>
+      <c r="AG20" s="56"/>
       <c r="AH20" s="7"/>
-      <c r="AI20" s="50" t="s">
+      <c r="AI20" s="54" t="s">
         <v>212</v>
       </c>
-      <c r="AJ20" s="51"/>
-      <c r="AK20" s="52"/>
-      <c r="AO20" s="50" t="s">
+      <c r="AJ20" s="55"/>
+      <c r="AK20" s="57"/>
+      <c r="AO20" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="AP20" s="51"/>
-      <c r="AQ20" s="58"/>
+      <c r="AP20" s="55"/>
+      <c r="AQ20" s="56"/>
       <c r="AR20" s="7"/>
-      <c r="AS20" s="50" t="s">
+      <c r="AS20" s="54" t="s">
         <v>212</v>
       </c>
-      <c r="AT20" s="51"/>
-      <c r="AU20" s="52"/>
+      <c r="AT20" s="55"/>
+      <c r="AU20" s="57"/>
     </row>
     <row r="21" spans="6:47" ht="29" thickBot="1" x14ac:dyDescent="0.25">
       <c r="AE21" s="31" t="s">
@@ -8018,10 +8018,10 @@
     <row r="23" spans="6:47" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="25" spans="6:47" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="6:47" x14ac:dyDescent="0.2">
-      <c r="AE26" s="56" t="s">
+      <c r="AE26" s="49" t="s">
         <v>226</v>
       </c>
-      <c r="AF26" s="57"/>
+      <c r="AF26" s="50"/>
     </row>
     <row r="27" spans="6:47" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="AE27" s="28" t="s">
@@ -8079,13 +8079,6 @@
     </sortState>
   </autoFilter>
   <mergeCells count="16">
-    <mergeCell ref="AE26:AF26"/>
-    <mergeCell ref="AO13:AU13"/>
-    <mergeCell ref="AO14:AQ14"/>
-    <mergeCell ref="AS14:AU14"/>
-    <mergeCell ref="AO19:AU19"/>
-    <mergeCell ref="AO20:AQ20"/>
-    <mergeCell ref="AS20:AU20"/>
     <mergeCell ref="N1:W1"/>
     <mergeCell ref="Y1:AH1"/>
     <mergeCell ref="AI14:AK14"/>
@@ -8095,6 +8088,13 @@
     <mergeCell ref="AJ5:AK5"/>
     <mergeCell ref="AE20:AG20"/>
     <mergeCell ref="AE14:AG14"/>
+    <mergeCell ref="AE26:AF26"/>
+    <mergeCell ref="AO13:AU13"/>
+    <mergeCell ref="AO14:AQ14"/>
+    <mergeCell ref="AS14:AU14"/>
+    <mergeCell ref="AO19:AU19"/>
+    <mergeCell ref="AO20:AQ20"/>
+    <mergeCell ref="AS20:AU20"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="AE14">
@@ -8112,101 +8112,101 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE20">
-    <cfRule type="cellIs" dxfId="83" priority="89" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="92" operator="equal">
+      <formula>"++"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="82" priority="89" operator="equal">
       <formula>"--"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="90" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="90" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="91" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="91" operator="equal">
       <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="92" operator="equal">
-      <formula>"++"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE26:AF26">
-    <cfRule type="cellIs" dxfId="79" priority="41" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="79" priority="44" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="43" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="77" priority="42" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="43" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="44" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="76" priority="41" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE15:AG15">
-    <cfRule type="cellIs" dxfId="75" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="64" operator="equal">
+      <formula>"++"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="74" priority="61" operator="equal">
       <formula>"--"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="62" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="63" operator="equal">
       <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="64" operator="equal">
-      <formula>"++"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE21:AG21">
-    <cfRule type="cellIs" dxfId="71" priority="81" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="71" priority="84" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="83" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="69" priority="82" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="83" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="84" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="68" priority="81" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE13:AK13">
-    <cfRule type="cellIs" dxfId="67" priority="113" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="116" operator="equal">
+      <formula>"++"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="113" operator="equal">
       <formula>"--"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="114" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="114" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="115" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="115" operator="equal">
       <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="116" operator="equal">
-      <formula>"++"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE19:AK19">
-    <cfRule type="cellIs" dxfId="63" priority="93" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="63" priority="96" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="94" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="95" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="94" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="95" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="96" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="60" priority="93" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI14">
-    <cfRule type="cellIs" dxfId="59" priority="53" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="59" priority="56" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="55" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="57" priority="54" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="55" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="56" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="56" priority="53" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI20">
@@ -8224,98 +8224,98 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI15:AK15">
-    <cfRule type="cellIs" dxfId="51" priority="49" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="51" priority="52" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="51" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="50" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="51" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="52" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="48" priority="49" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI21:AK21">
-    <cfRule type="cellIs" dxfId="47" priority="57" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="47" priority="60" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="58" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="59" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="58" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="59" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="60" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="44" priority="57" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ5:AK5">
     <cfRule type="cellIs" dxfId="43" priority="45" operator="equal">
       <formula>"--"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="46" operator="equal">
-      <formula>"-"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="47" operator="equal">
       <formula>"+"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="48" operator="equal">
       <formula>"++"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="46" operator="equal">
+      <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO14">
-    <cfRule type="cellIs" dxfId="39" priority="33" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="39" priority="36" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="35" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="34" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="35" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="36" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="36" priority="33" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO20">
-    <cfRule type="cellIs" dxfId="35" priority="13" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="35" priority="16" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="15" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="14" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="15" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="16" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="32" priority="13" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO15:AQ15">
-    <cfRule type="cellIs" dxfId="31" priority="29" operator="equal">
-      <formula>"--"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="30" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="31" operator="equal">
       <formula>"+"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="32" operator="equal">
       <formula>"++"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="29" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO21:AQ21">
-    <cfRule type="cellIs" dxfId="27" priority="9" operator="equal">
-      <formula>"--"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="10" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="11" operator="equal">
       <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="9" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="24" priority="12" operator="equal">
       <formula>"++"</formula>
@@ -8336,25 +8336,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO19:AU19">
-    <cfRule type="cellIs" dxfId="19" priority="17" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="19" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="18" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="19" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="20" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AS14">
-    <cfRule type="cellIs" dxfId="15" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="26" operator="equal">
+      <formula>"-"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="25" operator="equal">
       <formula>"--"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="26" operator="equal">
-      <formula>"-"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="13" priority="27" operator="equal">
       <formula>"+"</formula>
@@ -8364,25 +8364,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AS20">
-    <cfRule type="cellIs" dxfId="11" priority="5" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
+      <formula>"+"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
-      <formula>"+"</formula>
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
       <formula>"++"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AS15:AU15">
-    <cfRule type="cellIs" dxfId="7" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="22" operator="equal">
+      <formula>"-"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="21" operator="equal">
       <formula>"--"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="22" operator="equal">
-      <formula>"-"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="5" priority="23" operator="equal">
       <formula>"+"</formula>
@@ -8392,17 +8392,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AS21:AU21">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
-      <formula>"--"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"++"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"+"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"-"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
-      <formula>"+"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
-      <formula>"++"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"--"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>